<commit_message>
aggiornamento test 448, 449
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#NETHICALSRLXX/NETHICAL/NETHICAL_SRL/1.0.0/accreditamento-checklist_V9.0.0.xlsx
+++ b/GATEWAY/A1#111#NETHICALSRLXX/NETHICAL/NETHICAL_SRL/1.0.0/accreditamento-checklist_V9.0.0.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emanuele\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emanuele\it-fse-accreditamento\GATEWAY\A1#111#NETHICALSRLXX\NETHICAL\NETHICAL_SRL\1.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EB6AF7A-FA15-49D3-91D7-E025DF571D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B14C2CA-EC58-4397-A4BD-3FB0575C145A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43110" yWindow="0" windowWidth="14595" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -24,21 +24,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Summary!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TestCases!$A$9:$W$285</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="oXWj5iU3LtnvLpdhFqszSz/X91q3fG5U5zC5TJKtiGw="/>
@@ -2491,24 +2480,6 @@
     <t>Errore vocabolario : [http status code 400 ] - Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.6.1 v2.80, Codes: 60975000-0]</t>
   </si>
   <si>
-    <t>2026-02-11T12:22:22</t>
-  </si>
-  <si>
-    <t>ede6fa96cb67681f77fa1705e25e611c</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.deec95f5683dc06217a244ca42693cf5d43037c9d949711440c2ec0d7b7c1b85.c395035ae8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-02-11T12:09:08</t>
-  </si>
-  <si>
-    <t>0f14073592f8e47dd77036d3383bed4e</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.c460380a6b91a9acfd22762f448cc003ae12762aa890d63bbdac1485bfaba1a3.7306a51de7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-02-11T15:11:53</t>
   </si>
   <si>
@@ -2729,6 +2700,24 @@
   </si>
   <si>
     <t>Compare a video all'operatore il seguente messaggio: L'operazione è stata annullata o ha impiegato troppo tempo.</t>
+  </si>
+  <si>
+    <t>2026-03-25T12:30:04</t>
+  </si>
+  <si>
+    <t>35ab2b4b2850ecf7a18aa8a746609c26</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.76942b81f8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-25T12:27:37</t>
+  </si>
+  <si>
+    <t>e1a02e2003dd124a65cdd35759abf90e</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.4cb78cdbc0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -3476,6 +3465,16 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3498,16 +3497,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{565105C8-FFD6-432C-8B2E-BD1D172FCD26}"/>
@@ -4961,7 +4950,7 @@
     <col min="6" max="9" width="33.21875" customWidth="1"/>
     <col min="10" max="10" width="27.21875" customWidth="1"/>
     <col min="11" max="18" width="36.44140625" customWidth="1"/>
-    <col min="19" max="19" width="27.21875" style="79" customWidth="1"/>
+    <col min="19" max="19" width="27.21875" style="67" customWidth="1"/>
     <col min="20" max="20" width="33.21875" customWidth="1"/>
     <col min="21" max="21" width="36.44140625" customWidth="1"/>
     <col min="22" max="23" width="31.77734375" customWidth="1"/>
@@ -4983,19 +4972,19 @@
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="7"/>
-      <c r="S1" s="76"/>
+      <c r="S1" s="64"/>
       <c r="T1" s="7"/>
       <c r="U1" s="8"/>
       <c r="V1" s="2"/>
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="67"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="71"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -5009,21 +4998,21 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
-      <c r="S2" s="76"/>
+      <c r="S2" s="64"/>
       <c r="T2" s="7"/>
       <c r="U2" s="8"/>
       <c r="V2" s="2"/>
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="75" t="s">
+      <c r="B3" s="74"/>
+      <c r="C3" s="79" t="s">
         <v>629</v>
       </c>
-      <c r="D3" s="67"/>
+      <c r="D3" s="71"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -5037,19 +5026,19 @@
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
-      <c r="S3" s="76"/>
+      <c r="S3" s="64"/>
       <c r="T3" s="7"/>
       <c r="U3" s="8"/>
       <c r="V3" s="2"/>
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="71"/>
-      <c r="B4" s="72"/>
-      <c r="C4" s="75" t="s">
+      <c r="A4" s="75"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="79" t="s">
         <v>630</v>
       </c>
-      <c r="D4" s="67"/>
+      <c r="D4" s="71"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -5064,19 +5053,19 @@
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
-      <c r="S4" s="76"/>
+      <c r="S4" s="64"/>
       <c r="T4" s="7"/>
       <c r="U4" s="8"/>
       <c r="V4" s="2"/>
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="73"/>
-      <c r="B5" s="74"/>
-      <c r="C5" s="75" t="s">
+      <c r="A5" s="77"/>
+      <c r="B5" s="78"/>
+      <c r="C5" s="79" t="s">
         <v>631</v>
       </c>
-      <c r="D5" s="67"/>
+      <c r="D5" s="71"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -5090,15 +5079,15 @@
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
-      <c r="S5" s="76"/>
+      <c r="S5" s="64"/>
       <c r="T5" s="7"/>
       <c r="U5" s="8"/>
       <c r="V5" s="2"/>
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="64"/>
-      <c r="B6" s="65"/>
+      <c r="A6" s="68"/>
+      <c r="B6" s="69"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -5113,7 +5102,7 @@
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
-      <c r="S6" s="76"/>
+      <c r="S6" s="64"/>
       <c r="T6" s="7"/>
       <c r="U6" s="8"/>
       <c r="V6" s="2"/>
@@ -5136,7 +5125,7 @@
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
-      <c r="S7" s="76"/>
+      <c r="S7" s="64"/>
       <c r="T7" s="7"/>
       <c r="U7" s="8"/>
       <c r="V7" s="2"/>
@@ -5156,7 +5145,7 @@
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
-      <c r="S8" s="76"/>
+      <c r="S8" s="64"/>
       <c r="T8" s="7"/>
       <c r="U8" s="8"/>
       <c r="V8" s="2"/>
@@ -5217,7 +5206,7 @@
       <c r="R9" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="S9" s="77" t="s">
+      <c r="S9" s="65" t="s">
         <v>37</v>
       </c>
       <c r="T9" s="17" t="s">
@@ -5469,7 +5458,7 @@
       <c r="R15" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S15" s="78" t="s">
+      <c r="S15" s="66" t="s">
         <v>638</v>
       </c>
       <c r="T15" s="32"/>
@@ -5789,7 +5778,7 @@
       <c r="R23" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S23" s="78" t="s">
+      <c r="S23" s="66" t="s">
         <v>638</v>
       </c>
       <c r="T23" s="32"/>
@@ -6098,7 +6087,7 @@
         <v>635</v>
       </c>
       <c r="O31" s="32" t="s">
-        <v>734</v>
+        <v>728</v>
       </c>
       <c r="P31" s="32" t="s">
         <v>635</v>
@@ -6109,8 +6098,8 @@
       <c r="R31" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S31" s="78" t="s">
-        <v>735</v>
+      <c r="S31" s="66" t="s">
+        <v>729</v>
       </c>
       <c r="T31" s="32"/>
       <c r="U31" s="33" t="s">
@@ -9255,13 +9244,13 @@
         <v>46064</v>
       </c>
       <c r="G116" s="31" t="s">
-        <v>729</v>
+        <v>723</v>
       </c>
       <c r="H116" s="31" t="s">
-        <v>730</v>
+        <v>724</v>
       </c>
       <c r="I116" s="36" t="s">
-        <v>731</v>
+        <v>725</v>
       </c>
       <c r="J116" s="32" t="s">
         <v>635</v>
@@ -9275,7 +9264,7 @@
         <v>635</v>
       </c>
       <c r="O116" s="32" t="s">
-        <v>732</v>
+        <v>726</v>
       </c>
       <c r="P116" s="32" t="s">
         <v>635</v>
@@ -9286,8 +9275,8 @@
       <c r="R116" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S116" s="78" t="s">
-        <v>733</v>
+      <c r="S116" s="66" t="s">
+        <v>727</v>
       </c>
       <c r="T116" s="32"/>
       <c r="U116" s="33"/>
@@ -9316,13 +9305,13 @@
         <v>46064</v>
       </c>
       <c r="G117" s="31" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
       <c r="H117" s="31" t="s">
-        <v>725</v>
+        <v>719</v>
       </c>
       <c r="I117" s="36" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="J117" s="32" t="s">
         <v>635</v>
@@ -9336,7 +9325,7 @@
         <v>635</v>
       </c>
       <c r="O117" s="32" t="s">
-        <v>727</v>
+        <v>721</v>
       </c>
       <c r="P117" s="32" t="s">
         <v>635</v>
@@ -9347,8 +9336,8 @@
       <c r="R117" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S117" s="78" t="s">
-        <v>728</v>
+      <c r="S117" s="66" t="s">
+        <v>722</v>
       </c>
       <c r="T117" s="32"/>
       <c r="U117" s="33"/>
@@ -9377,13 +9366,13 @@
         <v>46064</v>
       </c>
       <c r="G118" s="31" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="H118" s="31" t="s">
-        <v>720</v>
+        <v>714</v>
       </c>
       <c r="I118" s="36" t="s">
-        <v>721</v>
+        <v>715</v>
       </c>
       <c r="J118" s="32" t="s">
         <v>635</v>
@@ -9397,7 +9386,7 @@
         <v>635</v>
       </c>
       <c r="O118" s="32" t="s">
-        <v>722</v>
+        <v>716</v>
       </c>
       <c r="P118" s="32" t="s">
         <v>635</v>
@@ -9408,8 +9397,8 @@
       <c r="R118" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S118" s="78" t="s">
-        <v>723</v>
+      <c r="S118" s="66" t="s">
+        <v>717</v>
       </c>
       <c r="T118" s="32"/>
       <c r="U118" s="33"/>
@@ -9438,13 +9427,13 @@
         <v>46064</v>
       </c>
       <c r="G119" s="31" t="s">
-        <v>714</v>
+        <v>708</v>
       </c>
       <c r="H119" s="31" t="s">
-        <v>715</v>
+        <v>709</v>
       </c>
       <c r="I119" s="36" t="s">
-        <v>716</v>
+        <v>710</v>
       </c>
       <c r="J119" s="32" t="s">
         <v>635</v>
@@ -9458,7 +9447,7 @@
         <v>635</v>
       </c>
       <c r="O119" s="32" t="s">
-        <v>717</v>
+        <v>711</v>
       </c>
       <c r="P119" s="32" t="s">
         <v>635</v>
@@ -9469,8 +9458,8 @@
       <c r="R119" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S119" s="78" t="s">
-        <v>718</v>
+      <c r="S119" s="66" t="s">
+        <v>712</v>
       </c>
       <c r="T119" s="32"/>
       <c r="U119" s="33"/>
@@ -9499,13 +9488,13 @@
         <v>46064</v>
       </c>
       <c r="G120" s="31" t="s">
-        <v>710</v>
+        <v>704</v>
       </c>
       <c r="H120" s="31" t="s">
-        <v>711</v>
+        <v>705</v>
       </c>
       <c r="I120" s="36" t="s">
-        <v>712</v>
+        <v>706</v>
       </c>
       <c r="J120" s="32" t="s">
         <v>635</v>
@@ -9519,7 +9508,7 @@
         <v>635</v>
       </c>
       <c r="O120" s="32" t="s">
-        <v>713</v>
+        <v>707</v>
       </c>
       <c r="P120" s="32" t="s">
         <v>635</v>
@@ -9530,8 +9519,8 @@
       <c r="R120" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S120" s="78" t="s">
-        <v>709</v>
+      <c r="S120" s="66" t="s">
+        <v>703</v>
       </c>
       <c r="T120" s="32"/>
       <c r="U120" s="33"/>
@@ -9560,13 +9549,13 @@
         <v>46064</v>
       </c>
       <c r="G121" s="31" t="s">
-        <v>705</v>
+        <v>699</v>
       </c>
       <c r="H121" s="31" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="I121" s="36" t="s">
-        <v>707</v>
+        <v>701</v>
       </c>
       <c r="J121" s="32" t="s">
         <v>635</v>
@@ -9580,7 +9569,7 @@
         <v>635</v>
       </c>
       <c r="O121" s="32" t="s">
-        <v>708</v>
+        <v>702</v>
       </c>
       <c r="P121" s="32" t="s">
         <v>635</v>
@@ -9591,8 +9580,8 @@
       <c r="R121" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S121" s="78" t="s">
-        <v>709</v>
+      <c r="S121" s="66" t="s">
+        <v>703</v>
       </c>
       <c r="T121" s="32"/>
       <c r="U121" s="33"/>
@@ -9621,13 +9610,13 @@
         <v>46064</v>
       </c>
       <c r="G122" s="31" t="s">
-        <v>700</v>
+        <v>694</v>
       </c>
       <c r="H122" s="31" t="s">
-        <v>701</v>
+        <v>695</v>
       </c>
       <c r="I122" s="36" t="s">
-        <v>702</v>
+        <v>696</v>
       </c>
       <c r="J122" s="32" t="s">
         <v>635</v>
@@ -9641,7 +9630,7 @@
         <v>635</v>
       </c>
       <c r="O122" s="32" t="s">
-        <v>703</v>
+        <v>697</v>
       </c>
       <c r="P122" s="32" t="s">
         <v>635</v>
@@ -9652,8 +9641,8 @@
       <c r="R122" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S122" s="78" t="s">
-        <v>704</v>
+      <c r="S122" s="66" t="s">
+        <v>698</v>
       </c>
       <c r="T122" s="32"/>
       <c r="U122" s="33"/>
@@ -9682,13 +9671,13 @@
         <v>46064</v>
       </c>
       <c r="G123" s="31" t="s">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="H123" s="31" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="I123" s="36" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
       <c r="J123" s="32" t="s">
         <v>635</v>
@@ -9702,7 +9691,7 @@
         <v>635</v>
       </c>
       <c r="O123" s="32" t="s">
-        <v>698</v>
+        <v>692</v>
       </c>
       <c r="P123" s="32" t="s">
         <v>635</v>
@@ -9713,8 +9702,8 @@
       <c r="R123" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S123" s="78" t="s">
-        <v>699</v>
+      <c r="S123" s="66" t="s">
+        <v>693</v>
       </c>
       <c r="T123" s="32"/>
       <c r="U123" s="33"/>
@@ -9743,13 +9732,13 @@
         <v>46064</v>
       </c>
       <c r="G124" s="31" t="s">
-        <v>690</v>
+        <v>684</v>
       </c>
       <c r="H124" s="31" t="s">
-        <v>691</v>
+        <v>685</v>
       </c>
       <c r="I124" s="36" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="J124" s="32" t="s">
         <v>635</v>
@@ -9763,7 +9752,7 @@
         <v>635</v>
       </c>
       <c r="O124" s="32" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
       <c r="P124" s="32" t="s">
         <v>635</v>
@@ -9774,8 +9763,8 @@
       <c r="R124" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S124" s="78" t="s">
-        <v>694</v>
+      <c r="S124" s="66" t="s">
+        <v>688</v>
       </c>
       <c r="T124" s="32"/>
       <c r="U124" s="33"/>
@@ -9804,13 +9793,13 @@
         <v>46064</v>
       </c>
       <c r="G125" s="31" t="s">
-        <v>686</v>
+        <v>680</v>
       </c>
       <c r="H125" s="31" t="s">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="I125" s="36" t="s">
-        <v>688</v>
+        <v>682</v>
       </c>
       <c r="J125" s="32" t="s">
         <v>635</v>
@@ -9824,7 +9813,7 @@
         <v>635</v>
       </c>
       <c r="O125" s="32" t="s">
-        <v>689</v>
+        <v>683</v>
       </c>
       <c r="P125" s="32" t="s">
         <v>635</v>
@@ -9835,8 +9824,8 @@
       <c r="R125" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S125" s="78" t="s">
-        <v>685</v>
+      <c r="S125" s="66" t="s">
+        <v>679</v>
       </c>
       <c r="T125" s="32"/>
       <c r="U125" s="33"/>
@@ -9865,13 +9854,13 @@
         <v>46064</v>
       </c>
       <c r="G126" s="31" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="H126" s="31" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="I126" s="36" t="s">
-        <v>683</v>
+        <v>677</v>
       </c>
       <c r="J126" s="32" t="s">
         <v>635</v>
@@ -9885,7 +9874,7 @@
         <v>635</v>
       </c>
       <c r="O126" s="32" t="s">
-        <v>684</v>
+        <v>678</v>
       </c>
       <c r="P126" s="32" t="s">
         <v>635</v>
@@ -9896,8 +9885,8 @@
       <c r="R126" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S126" s="78" t="s">
-        <v>685</v>
+      <c r="S126" s="66" t="s">
+        <v>679</v>
       </c>
       <c r="T126" s="32"/>
       <c r="U126" s="33"/>
@@ -9926,13 +9915,13 @@
         <v>46064</v>
       </c>
       <c r="G127" s="31" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
       <c r="H127" s="31" t="s">
-        <v>678</v>
+        <v>672</v>
       </c>
       <c r="I127" s="36" t="s">
-        <v>679</v>
+        <v>673</v>
       </c>
       <c r="J127" s="32" t="s">
         <v>635</v>
@@ -9946,7 +9935,7 @@
         <v>635</v>
       </c>
       <c r="O127" s="32" t="s">
-        <v>680</v>
+        <v>674</v>
       </c>
       <c r="P127" s="32" t="s">
         <v>635</v>
@@ -9957,8 +9946,8 @@
       <c r="R127" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S127" s="78" t="s">
-        <v>676</v>
+      <c r="S127" s="66" t="s">
+        <v>670</v>
       </c>
       <c r="T127" s="32"/>
       <c r="U127" s="33"/>
@@ -9987,13 +9976,13 @@
         <v>46064</v>
       </c>
       <c r="G128" s="31" t="s">
-        <v>672</v>
+        <v>666</v>
       </c>
       <c r="H128" s="31" t="s">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="I128" s="36" t="s">
-        <v>674</v>
+        <v>668</v>
       </c>
       <c r="J128" s="32" t="s">
         <v>635</v>
@@ -10007,7 +9996,7 @@
         <v>635</v>
       </c>
       <c r="O128" s="32" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="P128" s="32" t="s">
         <v>635</v>
@@ -10018,8 +10007,8 @@
       <c r="R128" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S128" s="78" t="s">
-        <v>676</v>
+      <c r="S128" s="66" t="s">
+        <v>670</v>
       </c>
       <c r="T128" s="32"/>
       <c r="U128" s="33"/>
@@ -10048,13 +10037,13 @@
         <v>46064</v>
       </c>
       <c r="G129" s="31" t="s">
-        <v>667</v>
+        <v>661</v>
       </c>
       <c r="H129" s="60" t="s">
-        <v>668</v>
+        <v>662</v>
       </c>
       <c r="I129" s="36" t="s">
-        <v>669</v>
+        <v>663</v>
       </c>
       <c r="J129" s="32" t="s">
         <v>635</v>
@@ -10068,7 +10057,7 @@
         <v>635</v>
       </c>
       <c r="O129" s="32" t="s">
-        <v>670</v>
+        <v>664</v>
       </c>
       <c r="P129" s="32" t="s">
         <v>635</v>
@@ -10079,8 +10068,8 @@
       <c r="R129" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S129" s="78" t="s">
-        <v>671</v>
+      <c r="S129" s="66" t="s">
+        <v>665</v>
       </c>
       <c r="T129" s="32"/>
       <c r="U129" s="33"/>
@@ -10109,13 +10098,13 @@
         <v>46064</v>
       </c>
       <c r="G130" s="31" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="H130" s="31" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
       <c r="I130" s="36" t="s">
-        <v>664</v>
+        <v>658</v>
       </c>
       <c r="J130" s="32" t="s">
         <v>635</v>
@@ -10129,7 +10118,7 @@
         <v>635</v>
       </c>
       <c r="O130" s="32" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="P130" s="32" t="s">
         <v>635</v>
@@ -10140,8 +10129,8 @@
       <c r="R130" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S130" s="78" t="s">
-        <v>666</v>
+      <c r="S130" s="66" t="s">
+        <v>660</v>
       </c>
       <c r="T130" s="32"/>
       <c r="U130" s="33"/>
@@ -11390,18 +11379,18 @@
         <v>341</v>
       </c>
       <c r="F164" s="31">
-        <v>46064</v>
+        <v>46106</v>
       </c>
       <c r="G164" s="31" t="s">
-        <v>659</v>
+        <v>730</v>
       </c>
       <c r="H164" s="31" t="s">
-        <v>660</v>
+        <v>731</v>
       </c>
       <c r="I164" s="36" t="s">
-        <v>661</v>
-      </c>
-      <c r="J164" s="32" t="s">
+        <v>732</v>
+      </c>
+      <c r="J164" s="66" t="s">
         <v>635</v>
       </c>
       <c r="K164" s="32"/>
@@ -11412,7 +11401,7 @@
       <c r="P164" s="32"/>
       <c r="Q164" s="32"/>
       <c r="R164" s="32"/>
-      <c r="S164" s="78"/>
+      <c r="S164" s="66"/>
       <c r="T164" s="32"/>
       <c r="U164" s="33"/>
       <c r="V164" s="34"/>
@@ -11437,16 +11426,16 @@
         <v>343</v>
       </c>
       <c r="F165" s="31">
-        <v>46064</v>
+        <v>46106</v>
       </c>
       <c r="G165" s="31" t="s">
-        <v>656</v>
+        <v>733</v>
       </c>
       <c r="H165" s="31" t="s">
-        <v>657</v>
+        <v>734</v>
       </c>
       <c r="I165" s="36" t="s">
-        <v>658</v>
+        <v>735</v>
       </c>
       <c r="J165" s="32" t="s">
         <v>635</v>
@@ -11459,7 +11448,7 @@
       <c r="P165" s="32"/>
       <c r="Q165" s="32"/>
       <c r="R165" s="32"/>
-      <c r="S165" s="78"/>
+      <c r="S165" s="66"/>
       <c r="T165" s="32"/>
       <c r="U165" s="33"/>
       <c r="V165" s="34"/>
@@ -11888,7 +11877,7 @@
       <c r="R176" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S176" s="78" t="s">
+      <c r="S176" s="66" t="s">
         <v>646</v>
       </c>
       <c r="T176" s="32"/>
@@ -12171,7 +12160,7 @@
       <c r="R183" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S183" s="78" t="s">
+      <c r="S183" s="66" t="s">
         <v>651</v>
       </c>
       <c r="T183" s="32"/>
@@ -12454,7 +12443,7 @@
       <c r="R190" s="32" t="s">
         <v>637</v>
       </c>
-      <c r="S190" s="78" t="s">
+      <c r="S190" s="66" t="s">
         <v>646</v>
       </c>
       <c r="T190" s="32"/>
@@ -16005,7 +15994,7 @@
       <c r="P286" s="7"/>
       <c r="Q286" s="7"/>
       <c r="R286" s="7"/>
-      <c r="S286" s="76"/>
+      <c r="S286" s="64"/>
       <c r="T286" s="7"/>
       <c r="U286" s="8"/>
       <c r="V286" s="2"/>
@@ -16025,7 +16014,7 @@
       <c r="P287" s="7"/>
       <c r="Q287" s="7"/>
       <c r="R287" s="7"/>
-      <c r="S287" s="76"/>
+      <c r="S287" s="64"/>
       <c r="T287" s="7"/>
       <c r="U287" s="8"/>
       <c r="V287" s="2"/>
@@ -16045,7 +16034,7 @@
       <c r="P288" s="7"/>
       <c r="Q288" s="7"/>
       <c r="R288" s="7"/>
-      <c r="S288" s="76"/>
+      <c r="S288" s="64"/>
       <c r="T288" s="7"/>
       <c r="U288" s="8"/>
       <c r="V288" s="2"/>
@@ -16065,7 +16054,7 @@
       <c r="P289" s="7"/>
       <c r="Q289" s="7"/>
       <c r="R289" s="7"/>
-      <c r="S289" s="76"/>
+      <c r="S289" s="64"/>
       <c r="T289" s="7"/>
       <c r="U289" s="8"/>
       <c r="V289" s="2"/>
@@ -16085,7 +16074,7 @@
       <c r="P290" s="7"/>
       <c r="Q290" s="7"/>
       <c r="R290" s="7"/>
-      <c r="S290" s="76"/>
+      <c r="S290" s="64"/>
       <c r="T290" s="7"/>
       <c r="U290" s="8"/>
       <c r="V290" s="2"/>
@@ -16105,7 +16094,7 @@
       <c r="P291" s="7"/>
       <c r="Q291" s="7"/>
       <c r="R291" s="7"/>
-      <c r="S291" s="76"/>
+      <c r="S291" s="64"/>
       <c r="T291" s="7"/>
       <c r="U291" s="8"/>
       <c r="V291" s="2"/>
@@ -16125,7 +16114,7 @@
       <c r="P292" s="7"/>
       <c r="Q292" s="7"/>
       <c r="R292" s="7"/>
-      <c r="S292" s="76"/>
+      <c r="S292" s="64"/>
       <c r="T292" s="7"/>
       <c r="U292" s="8"/>
       <c r="V292" s="2"/>
@@ -16145,7 +16134,7 @@
       <c r="P293" s="7"/>
       <c r="Q293" s="7"/>
       <c r="R293" s="7"/>
-      <c r="S293" s="76"/>
+      <c r="S293" s="64"/>
       <c r="T293" s="7"/>
       <c r="U293" s="8"/>
       <c r="V293" s="2"/>
@@ -16165,7 +16154,7 @@
       <c r="P294" s="7"/>
       <c r="Q294" s="7"/>
       <c r="R294" s="7"/>
-      <c r="S294" s="76"/>
+      <c r="S294" s="64"/>
       <c r="T294" s="7"/>
       <c r="U294" s="8"/>
       <c r="V294" s="2"/>
@@ -16185,7 +16174,7 @@
       <c r="P295" s="7"/>
       <c r="Q295" s="7"/>
       <c r="R295" s="7"/>
-      <c r="S295" s="76"/>
+      <c r="S295" s="64"/>
       <c r="T295" s="7"/>
       <c r="U295" s="8"/>
       <c r="V295" s="2"/>
@@ -16205,7 +16194,7 @@
       <c r="P296" s="7"/>
       <c r="Q296" s="7"/>
       <c r="R296" s="7"/>
-      <c r="S296" s="76"/>
+      <c r="S296" s="64"/>
       <c r="T296" s="7"/>
       <c r="U296" s="8"/>
       <c r="V296" s="2"/>
@@ -16225,7 +16214,7 @@
       <c r="P297" s="7"/>
       <c r="Q297" s="7"/>
       <c r="R297" s="7"/>
-      <c r="S297" s="76"/>
+      <c r="S297" s="64"/>
       <c r="T297" s="7"/>
       <c r="U297" s="8"/>
       <c r="V297" s="2"/>
@@ -16245,7 +16234,7 @@
       <c r="P298" s="7"/>
       <c r="Q298" s="7"/>
       <c r="R298" s="7"/>
-      <c r="S298" s="76"/>
+      <c r="S298" s="64"/>
       <c r="T298" s="7"/>
       <c r="U298" s="8"/>
       <c r="V298" s="2"/>
@@ -16265,7 +16254,7 @@
       <c r="P299" s="7"/>
       <c r="Q299" s="7"/>
       <c r="R299" s="7"/>
-      <c r="S299" s="76"/>
+      <c r="S299" s="64"/>
       <c r="T299" s="7"/>
       <c r="U299" s="8"/>
       <c r="V299" s="2"/>
@@ -16285,7 +16274,7 @@
       <c r="P300" s="7"/>
       <c r="Q300" s="7"/>
       <c r="R300" s="7"/>
-      <c r="S300" s="76"/>
+      <c r="S300" s="64"/>
       <c r="T300" s="7"/>
       <c r="U300" s="8"/>
       <c r="V300" s="2"/>
@@ -16305,7 +16294,7 @@
       <c r="P301" s="7"/>
       <c r="Q301" s="7"/>
       <c r="R301" s="7"/>
-      <c r="S301" s="76"/>
+      <c r="S301" s="64"/>
       <c r="T301" s="7"/>
       <c r="U301" s="8"/>
       <c r="V301" s="2"/>
@@ -16325,7 +16314,7 @@
       <c r="P302" s="7"/>
       <c r="Q302" s="7"/>
       <c r="R302" s="7"/>
-      <c r="S302" s="76"/>
+      <c r="S302" s="64"/>
       <c r="T302" s="7"/>
       <c r="U302" s="8"/>
       <c r="V302" s="2"/>
@@ -16345,7 +16334,7 @@
       <c r="P303" s="7"/>
       <c r="Q303" s="7"/>
       <c r="R303" s="7"/>
-      <c r="S303" s="76"/>
+      <c r="S303" s="64"/>
       <c r="T303" s="7"/>
       <c r="U303" s="8"/>
       <c r="V303" s="2"/>
@@ -16365,7 +16354,7 @@
       <c r="P304" s="7"/>
       <c r="Q304" s="7"/>
       <c r="R304" s="7"/>
-      <c r="S304" s="76"/>
+      <c r="S304" s="64"/>
       <c r="T304" s="7"/>
       <c r="U304" s="8"/>
       <c r="V304" s="2"/>
@@ -16385,7 +16374,7 @@
       <c r="P305" s="7"/>
       <c r="Q305" s="7"/>
       <c r="R305" s="7"/>
-      <c r="S305" s="76"/>
+      <c r="S305" s="64"/>
       <c r="T305" s="7"/>
       <c r="U305" s="8"/>
       <c r="V305" s="2"/>
@@ -16405,7 +16394,7 @@
       <c r="P306" s="7"/>
       <c r="Q306" s="7"/>
       <c r="R306" s="7"/>
-      <c r="S306" s="76"/>
+      <c r="S306" s="64"/>
       <c r="T306" s="7"/>
       <c r="U306" s="8"/>
       <c r="V306" s="2"/>
@@ -16425,7 +16414,7 @@
       <c r="P307" s="7"/>
       <c r="Q307" s="7"/>
       <c r="R307" s="7"/>
-      <c r="S307" s="76"/>
+      <c r="S307" s="64"/>
       <c r="T307" s="7"/>
       <c r="U307" s="8"/>
       <c r="V307" s="2"/>
@@ -16445,7 +16434,7 @@
       <c r="P308" s="7"/>
       <c r="Q308" s="7"/>
       <c r="R308" s="7"/>
-      <c r="S308" s="76"/>
+      <c r="S308" s="64"/>
       <c r="T308" s="7"/>
       <c r="U308" s="8"/>
       <c r="V308" s="2"/>
@@ -16465,7 +16454,7 @@
       <c r="P309" s="7"/>
       <c r="Q309" s="7"/>
       <c r="R309" s="7"/>
-      <c r="S309" s="76"/>
+      <c r="S309" s="64"/>
       <c r="T309" s="7"/>
       <c r="U309" s="8"/>
       <c r="V309" s="2"/>
@@ -16485,7 +16474,7 @@
       <c r="P310" s="7"/>
       <c r="Q310" s="7"/>
       <c r="R310" s="7"/>
-      <c r="S310" s="76"/>
+      <c r="S310" s="64"/>
       <c r="T310" s="7"/>
       <c r="U310" s="8"/>
       <c r="V310" s="2"/>
@@ -16505,7 +16494,7 @@
       <c r="P311" s="7"/>
       <c r="Q311" s="7"/>
       <c r="R311" s="7"/>
-      <c r="S311" s="76"/>
+      <c r="S311" s="64"/>
       <c r="T311" s="7"/>
       <c r="U311" s="8"/>
       <c r="V311" s="2"/>
@@ -16525,7 +16514,7 @@
       <c r="P312" s="7"/>
       <c r="Q312" s="7"/>
       <c r="R312" s="7"/>
-      <c r="S312" s="76"/>
+      <c r="S312" s="64"/>
       <c r="T312" s="7"/>
       <c r="U312" s="8"/>
       <c r="V312" s="2"/>
@@ -16545,7 +16534,7 @@
       <c r="P313" s="7"/>
       <c r="Q313" s="7"/>
       <c r="R313" s="7"/>
-      <c r="S313" s="76"/>
+      <c r="S313" s="64"/>
       <c r="T313" s="7"/>
       <c r="U313" s="8"/>
       <c r="V313" s="2"/>
@@ -16565,7 +16554,7 @@
       <c r="P314" s="7"/>
       <c r="Q314" s="7"/>
       <c r="R314" s="7"/>
-      <c r="S314" s="76"/>
+      <c r="S314" s="64"/>
       <c r="T314" s="7"/>
       <c r="U314" s="8"/>
       <c r="V314" s="2"/>
@@ -16585,7 +16574,7 @@
       <c r="P315" s="7"/>
       <c r="Q315" s="7"/>
       <c r="R315" s="7"/>
-      <c r="S315" s="76"/>
+      <c r="S315" s="64"/>
       <c r="T315" s="7"/>
       <c r="U315" s="8"/>
       <c r="V315" s="2"/>
@@ -16605,7 +16594,7 @@
       <c r="P316" s="7"/>
       <c r="Q316" s="7"/>
       <c r="R316" s="7"/>
-      <c r="S316" s="76"/>
+      <c r="S316" s="64"/>
       <c r="T316" s="7"/>
       <c r="U316" s="8"/>
       <c r="V316" s="2"/>
@@ -16625,7 +16614,7 @@
       <c r="P317" s="7"/>
       <c r="Q317" s="7"/>
       <c r="R317" s="7"/>
-      <c r="S317" s="76"/>
+      <c r="S317" s="64"/>
       <c r="T317" s="7"/>
       <c r="U317" s="8"/>
       <c r="V317" s="2"/>
@@ -16645,7 +16634,7 @@
       <c r="P318" s="7"/>
       <c r="Q318" s="7"/>
       <c r="R318" s="7"/>
-      <c r="S318" s="76"/>
+      <c r="S318" s="64"/>
       <c r="T318" s="7"/>
       <c r="U318" s="8"/>
       <c r="V318" s="2"/>
@@ -16665,7 +16654,7 @@
       <c r="P319" s="7"/>
       <c r="Q319" s="7"/>
       <c r="R319" s="7"/>
-      <c r="S319" s="76"/>
+      <c r="S319" s="64"/>
       <c r="T319" s="7"/>
       <c r="U319" s="8"/>
       <c r="V319" s="2"/>
@@ -16685,7 +16674,7 @@
       <c r="P320" s="7"/>
       <c r="Q320" s="7"/>
       <c r="R320" s="7"/>
-      <c r="S320" s="76"/>
+      <c r="S320" s="64"/>
       <c r="T320" s="7"/>
       <c r="U320" s="8"/>
       <c r="V320" s="2"/>
@@ -16705,7 +16694,7 @@
       <c r="P321" s="7"/>
       <c r="Q321" s="7"/>
       <c r="R321" s="7"/>
-      <c r="S321" s="76"/>
+      <c r="S321" s="64"/>
       <c r="T321" s="7"/>
       <c r="U321" s="8"/>
       <c r="V321" s="2"/>
@@ -16725,7 +16714,7 @@
       <c r="P322" s="7"/>
       <c r="Q322" s="7"/>
       <c r="R322" s="7"/>
-      <c r="S322" s="76"/>
+      <c r="S322" s="64"/>
       <c r="T322" s="7"/>
       <c r="U322" s="8"/>
       <c r="V322" s="2"/>
@@ -16745,7 +16734,7 @@
       <c r="P323" s="7"/>
       <c r="Q323" s="7"/>
       <c r="R323" s="7"/>
-      <c r="S323" s="76"/>
+      <c r="S323" s="64"/>
       <c r="T323" s="7"/>
       <c r="U323" s="8"/>
       <c r="V323" s="2"/>
@@ -16765,7 +16754,7 @@
       <c r="P324" s="7"/>
       <c r="Q324" s="7"/>
       <c r="R324" s="7"/>
-      <c r="S324" s="76"/>
+      <c r="S324" s="64"/>
       <c r="T324" s="7"/>
       <c r="U324" s="8"/>
       <c r="V324" s="2"/>
@@ -16785,7 +16774,7 @@
       <c r="P325" s="7"/>
       <c r="Q325" s="7"/>
       <c r="R325" s="7"/>
-      <c r="S325" s="76"/>
+      <c r="S325" s="64"/>
       <c r="T325" s="7"/>
       <c r="U325" s="8"/>
       <c r="V325" s="2"/>
@@ -16805,7 +16794,7 @@
       <c r="P326" s="7"/>
       <c r="Q326" s="7"/>
       <c r="R326" s="7"/>
-      <c r="S326" s="76"/>
+      <c r="S326" s="64"/>
       <c r="T326" s="7"/>
       <c r="U326" s="8"/>
       <c r="V326" s="2"/>
@@ -16825,7 +16814,7 @@
       <c r="P327" s="7"/>
       <c r="Q327" s="7"/>
       <c r="R327" s="7"/>
-      <c r="S327" s="76"/>
+      <c r="S327" s="64"/>
       <c r="T327" s="7"/>
       <c r="U327" s="8"/>
       <c r="V327" s="2"/>
@@ -16845,7 +16834,7 @@
       <c r="P328" s="7"/>
       <c r="Q328" s="7"/>
       <c r="R328" s="7"/>
-      <c r="S328" s="76"/>
+      <c r="S328" s="64"/>
       <c r="T328" s="7"/>
       <c r="U328" s="8"/>
       <c r="V328" s="2"/>
@@ -16865,7 +16854,7 @@
       <c r="P329" s="7"/>
       <c r="Q329" s="7"/>
       <c r="R329" s="7"/>
-      <c r="S329" s="76"/>
+      <c r="S329" s="64"/>
       <c r="T329" s="7"/>
       <c r="U329" s="8"/>
       <c r="V329" s="2"/>
@@ -16885,7 +16874,7 @@
       <c r="P330" s="7"/>
       <c r="Q330" s="7"/>
       <c r="R330" s="7"/>
-      <c r="S330" s="76"/>
+      <c r="S330" s="64"/>
       <c r="T330" s="7"/>
       <c r="U330" s="8"/>
       <c r="V330" s="2"/>
@@ -16905,7 +16894,7 @@
       <c r="P331" s="7"/>
       <c r="Q331" s="7"/>
       <c r="R331" s="7"/>
-      <c r="S331" s="76"/>
+      <c r="S331" s="64"/>
       <c r="T331" s="7"/>
       <c r="U331" s="8"/>
       <c r="V331" s="2"/>

</xml_diff>